<commit_message>
add oncokb citation + CIViC update
</commit_message>
<xml_diff>
--- a/data-raw/metadata_pharm_oncox.xlsx
+++ b/data-raw/metadata_pharm_oncox.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__pharmOncoX/pharmOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F08D14B-E091-C440-90F8-D0C5B52ED9B6}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A6B716-0EC3-EF43-9E9E-B500F8AD96AD}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2580" windowWidth="35840" windowHeight="19820" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
+    <workbookView xWindow="0" yWindow="2580" windowWidth="35840" windowHeight="19820" activeTab="1" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
   <sheets>
     <sheet name="compounds" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="64">
   <si>
     <t>source</t>
   </si>
@@ -197,6 +197,27 @@
   </si>
   <si>
     <t>26.02d</t>
+  </si>
+  <si>
+    <t>OncoKB</t>
+  </si>
+  <si>
+    <t>OncoKB: A Precision Oncology Knowledge Base</t>
+  </si>
+  <si>
+    <t>https://www.oncokb.org/</t>
+  </si>
+  <si>
+    <t>Chakravarty et al., JCO Precis Oncol 2017; 28890946</t>
+  </si>
+  <si>
+    <t>Restricted</t>
+  </si>
+  <si>
+    <t>https://www.oncokb.org/terms</t>
+  </si>
+  <si>
+    <t>oncokb</t>
   </si>
 </sst>
 </file>
@@ -740,7 +761,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{932642DA-7C44-1E43-949C-73113CAEBEC0}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="36.33203125" customWidth="1"/>
@@ -859,7 +880,7 @@
       <c r="B5" t="s">
         <v>51</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="2" t="s">
         <v>47</v>
       </c>
       <c r="D5" t="s">
@@ -876,6 +897,29 @@
       </c>
       <c r="H5" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H6" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -886,6 +930,8 @@
     <hyperlink ref="H2" r:id="rId4" xr:uid="{228722B7-C7B7-8546-9D31-5872CF76F140}"/>
     <hyperlink ref="H4" r:id="rId5" xr:uid="{205EBEF1-9903-5946-B084-25D8A43F8D47}"/>
     <hyperlink ref="H3" r:id="rId6" xr:uid="{6FCA3D4F-3899-BC4C-BAE2-AFE2A58325F8}"/>
+    <hyperlink ref="C5" r:id="rId7" xr:uid="{68DF46BF-065F-4C43-97EC-8557D64C9A01}"/>
+    <hyperlink ref="C6" r:id="rId8" xr:uid="{CAB238B4-0B78-1245-AFAA-0D6075CD2017}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Silence PubChem synonym read_tsv warnings about extra columns
Some PubChem alias strings contain embedded tab characters, making
readr see a 3rd column and warn. Adding .default = col_skip() to the
col_types spec silently discards any extra fields instead of warning.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-raw/metadata_pharm_oncox.xlsx
+++ b/data-raw/metadata_pharm_oncox.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__pharmOncoX/pharmOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A6B716-0EC3-EF43-9E9E-B500F8AD96AD}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D947F56D-BF7B-3A42-8FEE-A8022627C119}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2580" windowWidth="35840" windowHeight="19820" activeTab="1" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
+    <workbookView xWindow="0" yWindow="2580" windowWidth="35840" windowHeight="19820" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
   <sheets>
     <sheet name="compounds" sheetId="2" r:id="rId1"/>
@@ -184,21 +184,12 @@
     <t>The Cancer Dependency Map</t>
   </si>
   <si>
-    <t>25Q3</t>
-  </si>
-  <si>
     <t>v2025</t>
   </si>
   <si>
     <t>2025.12</t>
   </si>
   <si>
-    <t>v20260115</t>
-  </si>
-  <si>
-    <t>26.02d</t>
-  </si>
-  <si>
     <t>OncoKB</t>
   </si>
   <si>
@@ -218,6 +209,15 @@
   </si>
   <si>
     <t>oncokb</t>
+  </si>
+  <si>
+    <t>26Q1</t>
+  </si>
+  <si>
+    <t>v20260415</t>
+  </si>
+  <si>
+    <t>26.04d</t>
   </si>
 </sst>
 </file>
@@ -681,7 +681,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -707,7 +707,7 @@
         <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="F3" t="s">
         <v>9</v>
@@ -733,7 +733,7 @@
         <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F4" t="s">
         <v>13</v>
@@ -835,7 +835,7 @@
         <v>18</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>19</v>
@@ -887,7 +887,7 @@
         <v>48</v>
       </c>
       <c r="E5" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="F5" t="s">
         <v>46</v>
@@ -901,25 +901,25 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" t="s">
         <v>57</v>
       </c>
-      <c r="B6" t="s">
+      <c r="F6" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" t="s">
         <v>58</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="H6" t="s">
         <v>59</v>
-      </c>
-      <c r="D6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="G6" t="s">
-        <v>61</v>
-      </c>
-      <c r="H6" t="s">
-        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
OTP 2026.03, NCI thes 26.04d, QMD vignette
</commit_message>
<xml_diff>
--- a/data-raw/metadata_pharm_oncox.xlsx
+++ b/data-raw/metadata_pharm_oncox.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__pharmOncoX/pharmOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D947F56D-BF7B-3A42-8FEE-A8022627C119}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4976EF2-1314-4B47-9AE9-EDD596CC541B}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="2580" windowWidth="35840" windowHeight="19820" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
@@ -187,9 +187,6 @@
     <t>v2025</t>
   </si>
   <si>
-    <t>2025.12</t>
-  </si>
-  <si>
     <t>OncoKB</t>
   </si>
   <si>
@@ -218,6 +215,9 @@
   </si>
   <si>
     <t>26.04d</t>
+  </si>
+  <si>
+    <t>2026.03</t>
   </si>
 </sst>
 </file>
@@ -681,7 +681,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -707,7 +707,7 @@
         <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F3" t="s">
         <v>9</v>
@@ -835,7 +835,7 @@
         <v>18</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>19</v>
@@ -887,7 +887,7 @@
         <v>48</v>
       </c>
       <c r="E5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F5" t="s">
         <v>46</v>
@@ -901,25 +901,25 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" t="s">
         <v>54</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" t="s">
         <v>56</v>
       </c>
-      <c r="D6" t="s">
+      <c r="F6" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G6" t="s">
         <v>57</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>58</v>
-      </c>
-      <c r="H6" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update CIViC + NCI Thesaurus
</commit_message>
<xml_diff>
--- a/data-raw/metadata_pharm_oncox.xlsx
+++ b/data-raw/metadata_pharm_oncox.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__pharmOncoX/pharmOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4976EF2-1314-4B47-9AE9-EDD596CC541B}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21598626-8714-E64D-A6FB-B52EFBA7F603}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="2580" windowWidth="35840" windowHeight="19820" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
@@ -184,9 +184,6 @@
     <t>The Cancer Dependency Map</t>
   </si>
   <si>
-    <t>v2025</t>
-  </si>
-  <si>
     <t>OncoKB</t>
   </si>
   <si>
@@ -214,10 +211,13 @@
     <t>v20260415</t>
   </si>
   <si>
-    <t>26.04d</t>
-  </si>
-  <si>
     <t>2026.03</t>
+  </si>
+  <si>
+    <t>26.05d</t>
+  </si>
+  <si>
+    <t>v2026</t>
   </si>
 </sst>
 </file>
@@ -681,7 +681,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -733,7 +733,7 @@
         <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="F4" t="s">
         <v>13</v>
@@ -835,7 +835,7 @@
         <v>18</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>19</v>
@@ -887,7 +887,7 @@
         <v>48</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F5" t="s">
         <v>46</v>
@@ -901,25 +901,25 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" t="s">
         <v>53</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" t="s">
         <v>55</v>
       </c>
-      <c r="D6" t="s">
+      <c r="F6" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="G6" t="s">
         <v>56</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>57</v>
-      </c>
-      <c r="H6" t="s">
-        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NCI Thesaurus 2026.06e, CIViC 20260708
</commit_message>
<xml_diff>
--- a/data-raw/metadata_pharm_oncox.xlsx
+++ b/data-raw/metadata_pharm_oncox.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__pharmOncoX/pharmOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21598626-8714-E64D-A6FB-B52EFBA7F603}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0255B300-AA62-8545-BD30-53333138FF6C}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2580" windowWidth="35840" windowHeight="19820" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
+    <workbookView xWindow="440" yWindow="1620" windowWidth="35840" windowHeight="19820" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
   <sheets>
     <sheet name="compounds" sheetId="2" r:id="rId1"/>
@@ -211,13 +211,13 @@
     <t>v20260415</t>
   </si>
   <si>
-    <t>2026.03</t>
-  </si>
-  <si>
-    <t>26.05d</t>
-  </si>
-  <si>
     <t>v2026</t>
+  </si>
+  <si>
+    <t>26.06e</t>
+  </si>
+  <si>
+    <t>2026.06</t>
   </si>
 </sst>
 </file>
@@ -681,7 +681,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -733,7 +733,7 @@
         <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F4" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
NCI Thesaurus 26.07d, Mitelmandb 20250715
</commit_message>
<xml_diff>
--- a/data-raw/metadata_pharm_oncox.xlsx
+++ b/data-raw/metadata_pharm_oncox.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__pharmOncoX/pharmOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0255B300-AA62-8545-BD30-53333138FF6C}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2CC4F3B-0E21-9247-81EA-F72D7C3DD024}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="440" yWindow="1620" windowWidth="35840" windowHeight="19820" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
+    <workbookView xWindow="0" yWindow="1620" windowWidth="35840" windowHeight="19820" activeTab="1" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
   <sheets>
     <sheet name="compounds" sheetId="2" r:id="rId1"/>
@@ -208,16 +208,16 @@
     <t>26Q1</t>
   </si>
   <si>
-    <t>v20260415</t>
-  </si>
-  <si>
     <t>v2026</t>
   </si>
   <si>
-    <t>26.06e</t>
-  </si>
-  <si>
     <t>2026.06</t>
+  </si>
+  <si>
+    <t>26.07d</t>
+  </si>
+  <si>
+    <t>v20260715</t>
   </si>
 </sst>
 </file>
@@ -681,7 +681,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -733,7 +733,7 @@
         <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F4" t="s">
         <v>13</v>
@@ -835,7 +835,7 @@
         <v>18</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
NCI Thesaurus 2026.08e, CIViC 20260903
</commit_message>
<xml_diff>
--- a/data-raw/metadata_pharm_oncox.xlsx
+++ b/data-raw/metadata_pharm_oncox.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sigven/project_data/packages/package__pharmOncoX/pharmOncoX/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2CC4F3B-0E21-9247-81EA-F72D7C3DD024}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00FFD2DA-EF72-B441-951D-A64BA7C9C1F3}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1620" windowWidth="35840" windowHeight="19820" activeTab="1" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
+    <workbookView xWindow="5160" yWindow="1620" windowWidth="35840" windowHeight="19820" xr2:uid="{FE925BBA-8697-304B-A498-CFC01A1CEF4E}"/>
   </bookViews>
   <sheets>
     <sheet name="compounds" sheetId="2" r:id="rId1"/>
@@ -214,10 +214,10 @@
     <t>2026.06</t>
   </si>
   <si>
-    <t>26.07d</t>
-  </si>
-  <si>
     <t>v20260715</t>
+  </si>
+  <si>
+    <t>26.08e</t>
   </si>
 </sst>
 </file>
@@ -707,7 +707,7 @@
         <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F3" t="s">
         <v>9</v>
@@ -835,7 +835,7 @@
         <v>18</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>19</v>

</xml_diff>